<commit_message>
feat(qc+l4): chemistry-anchored voltage windows, protocol-graded GITT QC, L4 rate-prediction acceptance
A 体系锚定电压窗: battery_sim/datasets/chemistry_windows.py (nominal/hard 两级,
闭集, 不猜声明) + user_tools/validate.py 两条新码 VOLTAGE_WINDOW_SYSTEM /
VOLTAGE_SYSTEM_RANGE; experiment 表新增 working_electrode_material.

B 脉冲协议 QC 分级: protocol_type 进闭集; 脉冲协议下采样间断升 FAIL;
新增 GITT_STRUCTURE / GITT_PULSE_DURATION (5% 容差) / GITT_PULSE_UNIFORMITY /
GITT_PULSE_RESOLUTION; 新增 pulse_duration_s / relax_duration_s (17 -> 21 字段).

C L4 倍率预测验收: identification/rate_prediction.py + 合成倍率梯夹具
examples/synthetic_rate_ladder/; 四道门 (角色 / 尺度 / 覆盖率 / 初值接线).
实测 真值 3.27 mV vs 零拟合负对照 20.09 mV.

修复: RecycledGraphiteAdapter.load_processed_discharge 未挂 attrs['initialisation']
-> 半电池 GCD 回放从参数集默认初值出发 (起点偏 708 mV, RMSE 被初值差吃掉);
同一夹具 59.89 -> 3.27 mV.

平台科学核心 (runner/evaluator/factory/registry/rates/paths) 改动 = 0.
tests: 549 -> 597 (test_user_data_qc 29 + test_rate_prediction 19).
</commit_message>
<xml_diff>
--- a/user_dataset_template/dataset_info.xlsx
+++ b/user_dataset_template/dataset_info.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -491,11 +491,7 @@
           <t>数据集名称</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>demo_birmingham_cover5</t>
-        </is>
-      </c>
+      <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr">
         <is>
           <t>必填</t>
@@ -513,11 +509,7 @@
           <t>样品编号</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>NCM920305_demo</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>必填</t>
@@ -535,11 +527,7 @@
           <t>正极化学体系</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>NMC</t>
-        </is>
-      </c>
+      <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
           <t>必填；只能填：LFP / NMC / LCO / other</t>
@@ -549,123 +537,105 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>cell_configuration</t>
+          <t>dataset_role</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>电池构型</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>half_cell</t>
-        </is>
-      </c>
+          <t>数据用途</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>必填；只能填：full_cell / half_cell</t>
+          <t>可选；只能填：identification / validation / benchmark / prediction</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>working_electrode</t>
+          <t>cell_configuration</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>工作电极</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
+          <t>电池构型</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">可选；只能填：positive / negative / </t>
+          <t>必填；只能填：full_cell / half_cell</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>counter_electrode</t>
+          <t>working_electrode</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>对电极</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>lithium_metal</t>
-        </is>
-      </c>
+          <t>工作电极</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">可选；只能填：lithium_metal / graphite / other / </t>
+          <t xml:space="preserve">可选；只能填：positive / negative / </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>nominal_capacity</t>
+          <t>working_electrode_material</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>标称容量 [Ah]</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.003112</v>
-      </c>
+          <t>工作电极材料</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t xml:space="preserve">可选；只能填：graphite / nmc / lfp / lco / lithium_metal / silicon_c / other / </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>active_material_loading</t>
+          <t>counter_electrode</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>面容量 [mAh/cm2]</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2</v>
-      </c>
+          <t>对电极</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t xml:space="preserve">可选；只能填：lithium_metal / graphite / other / </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>electrode_area</t>
+          <t>nominal_capacity</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>极片面积 [cm2]</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1.72</v>
-      </c>
+          <t>标称容量 [Ah]</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
           <t>可选</t>
@@ -675,19 +645,15 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>electrolyte</t>
+          <t>active_material_loading</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>电解液</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>LiPF6 (Celgard 2325)</t>
-        </is>
-      </c>
+          <t>面容量 [mAh/cm2]</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>可选</t>
@@ -697,116 +663,102 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>voltage_lower</t>
+          <t>electrode_area</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>下限电压 [V]</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>2.5</v>
-      </c>
+          <t>极片面积 [cm2]</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>必填</t>
+          <t>可选</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>voltage_upper</t>
+          <t>electrolyte</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>上限电压 [V]</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>4.2</v>
-      </c>
+          <t>电解液</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>必填</t>
+          <t>可选</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>voltage_lower</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>环境温度 [C]</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>25</v>
-      </c>
+          <t>下限电压 [V]</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>必填</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>protocol</t>
+          <t>voltage_upper</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>测试protocol</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CC_Cover5</t>
-        </is>
-      </c>
+          <t>上限电压 [V]</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>必填</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>current_sign</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>原始电流符号</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>discharge_negative</t>
-        </is>
-      </c>
+          <t>环境温度 [C]</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>必填；只能填：discharge_positive / discharge_negative</t>
+          <t>可选</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>initial_soc</t>
+          <t>protocol</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>初始 SOC (0-1, 可选)</t>
+          <t>测试protocol（原始档位名）</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -816,21 +768,120 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>protocol_type</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>协议类型（闭集）</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">可选；只能填：GCD / GITT / PITT / pOCV / rate_capability / cycle_life / EIS / other / </t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>pulse_duration_s</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>GITT 脉冲时长 [s]</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>relax_duration_s</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>GITT 静置时长 [s]</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>current_sign</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>原始电流符号</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>必填；只能填：discharge_positive / discharge_negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>initial_soc</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>初始 SOC (0-1, 可选)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="8">
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LFP,NMC,LCO,other"</formula1>
     </dataValidation>
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"identification,validation,benchmark,prediction"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"full_cell,half_cell"</formula1>
     </dataValidation>
-    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"positive,negative,"</formula1>
     </dataValidation>
-    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"graphite,nmc,lfp,lco,lithium_metal,silicon_c,other,"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"lithium_metal,graphite,other,"</formula1>
     </dataValidation>
-    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"GCD,GITT,PITT,pOCV,rate_capability,cycle_life,EIS,other,"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"discharge_positive,discharge_negative"</formula1>
     </dataValidation>
   </dataValidations>
@@ -892,16 +943,8 @@
           <t>时间</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Time [s]</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
           <t>必填；单位只能填：h / hour / min / ms / s / sec</t>
@@ -919,16 +962,8 @@
           <t>电流</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Current [mA]</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>mA</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>必填；单位只能填：a / ma / ua / µa</t>
@@ -946,16 +981,8 @@
           <t>电压</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Voltage [V]</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>必填；单位只能填：mv / v</t>
@@ -973,16 +1000,8 @@
           <t>容量</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Capacity [mAh]</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>mAh</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>可选；单位只能填：ah / mah</t>
@@ -1038,16 +1057,8 @@
           <t>温度</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Temperature [K]</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>可选；单位只能填：c / f / k</t>
@@ -1088,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1101,7 +1112,9 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1109,7 +1122,9 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
@@ -1120,7 +1135,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chemistry        填 LFP / NMC / LCO / other</t>
+          <t xml:space="preserve">   chemistry        填 LFP / NMC / LCO / other（这一栏装的是正极体系）</t>
         </is>
       </c>
     </row>
@@ -1141,107 +1156,178 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   counter_electrode    半电池才填：对电极（锂金属填 lithium_metal）</t>
+          <t xml:space="preserve">   working_electrode_material  被测电极是什么材料（石墨填 graphite）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   current_sign     看你的原始数据：放电那一段电流是正数还是负数</t>
+          <t xml:space="preserve">                    平台靠它决定该用哪个电压窗口；留空会跳过这项检查</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    discharge_positive = 放电记为正</t>
+          <t xml:space="preserve">                    例如石墨半电池的窗口是 0.005-1.5 V，填 [0.005, 15] 会被拦下</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    discharge_negative = 放电记为负（多数设备是这种）</t>
+          <t xml:space="preserve">   counter_electrode    半电池才填：对电极（锂金属填 lithium_metal）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   voltage_lower / voltage_upper   你实际用的电压窗口（V）</t>
+          <t xml:space="preserve">   current_sign     看你的原始数据：放电那一段电流是正数还是负数</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   active_material_loading   半电池一定要填（面容量 mAh/cm2）</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
+          <t xml:space="preserve">                    discharge_positive = 放电记为正</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    discharge_negative = 放电记为负（多数设备是这种）</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>第四步：填 column_mapping 表。</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   voltage_lower / voltage_upper   你实际用的电压窗口（V）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   source_column = 你数据文件里的列名（要一模一样，含空格和方括号）</t>
+          <t xml:space="preserve">   active_material_loading   半电池一定要填（面容量 mAh/cm2）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   source_unit   = 那一列的单位（从下拉里选）</t>
+          <t xml:space="preserve">   protocol         仪器上的档位名，原样填（例如 CC_Cover5）</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   time / current / voltage 三行必填，其余没有就留空</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
+          <t xml:space="preserve">   protocol_type    协议类型，从下拉选（GCD / GITT / pOCV / ...）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    填了 GITT：采样间断与脉冲时长不一致会直接判错误</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>第五步：双击「导入并检查数据.bat」，看 validation_report.html。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    因为 Ds 就是由脉冲时长算出来的</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   pulse_duration_s / relax_duration_s  GITT 的脉冲与静置时长（秒）</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>第六步：报告说可以仿真时，再双击「运行仿真.bat」。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    填了平台会拿实测值核对；不填只给警告</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>注意：</t>
+          <t>第四步：填 column_mapping 表。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   本工具不做拟合，不调参数。跑出来的 RMSE 只是差异大小的参考，</t>
+          <t xml:space="preserve">   source_column = 你数据文件里的列名（要一模一样，含空格和方括号）</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   source_unit   = 那一列的单位（从下拉里选）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   time / current / voltage 三行必填，其余没有就留空</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>第五步：双击「导入并检查数据.bat」，看 validation_report.html。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>第六步：报告说可以仿真时，再双击「运行仿真.bat」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>注意：</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   本工具不做拟合，不调参数。跑出来的 RMSE 只是差异大小的参考，</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">   不等于模型验证，也不等于找到了误差原因。</t>
         </is>

</xml_diff>